<commit_message>
Deployed 39936fe with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/NSI_Premiere/Classeur1.xlsx
+++ b/NSI_Premiere/Classeur1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\--- LYCEE ---\ENSEIGNEMENT_G\docs\NSI_Premiere\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{96501FBC-9563-4318-9791-3CBE7E9AB228}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{372F3D1D-9786-49D3-8E2A-AC0827F8B947}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="4" xr2:uid="{C3D69442-6D2C-43E5-8165-E9BA2FDD5BB6}"/>
+    <workbookView xWindow="10718" yWindow="0" windowWidth="10965" windowHeight="12863" activeTab="4" xr2:uid="{C3D69442-6D2C-43E5-8165-E9BA2FDD5BB6}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="213">
   <si>
     <r>
       <t>ThèmeContenus (Compétence)Capacités attendues &amp; CommentairesN° Activité</t>
@@ -968,6 +968,27 @@
   </si>
   <si>
     <t>15bis</t>
+  </si>
+  <si>
+    <t>LP01</t>
+  </si>
+  <si>
+    <t>LP06</t>
+  </si>
+  <si>
+    <t>LP02</t>
+  </si>
+  <si>
+    <t>LP03</t>
+  </si>
+  <si>
+    <t>LP04</t>
+  </si>
+  <si>
+    <t>LP05</t>
+  </si>
+  <si>
+    <t>LP07</t>
   </si>
 </sst>
 </file>
@@ -1011,12 +1032,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -1031,7 +1058,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1046,6 +1073,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2023,7 +2051,7 @@
     <col min="3" max="4" width="42.9296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:4" ht="41.65" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:4" ht="27.75" x14ac:dyDescent="0.45">
       <c r="A3" s="2" t="s">
         <v>50</v>
       </c>
@@ -2049,7 +2077,7 @@
       </c>
       <c r="D4" s="3"/>
     </row>
-    <row r="5" spans="1:4" ht="27.75" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:4" ht="27" x14ac:dyDescent="0.45">
       <c r="A5" s="2" t="s">
         <v>76</v>
       </c>
@@ -2061,7 +2089,7 @@
       </c>
       <c r="D5" s="3"/>
     </row>
-    <row r="6" spans="1:4" ht="27.75" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:4" ht="27" x14ac:dyDescent="0.45">
       <c r="A6" s="2" t="s">
         <v>76</v>
       </c>
@@ -2073,7 +2101,7 @@
       </c>
       <c r="D6" s="3"/>
     </row>
-    <row r="7" spans="1:4" ht="27.75" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:4" ht="27" x14ac:dyDescent="0.45">
       <c r="A7" s="2" t="s">
         <v>76</v>
       </c>
@@ -2085,7 +2113,7 @@
       </c>
       <c r="D7" s="3"/>
     </row>
-    <row r="8" spans="1:4" ht="27.75" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:4" ht="27" x14ac:dyDescent="0.45">
       <c r="A8" s="2" t="s">
         <v>76</v>
       </c>
@@ -2097,7 +2125,7 @@
       </c>
       <c r="D8" s="3"/>
     </row>
-    <row r="9" spans="1:4" ht="27.75" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:4" ht="27" x14ac:dyDescent="0.45">
       <c r="A9" s="2" t="s">
         <v>76</v>
       </c>
@@ -2109,7 +2137,7 @@
       </c>
       <c r="D9" s="3"/>
     </row>
-    <row r="10" spans="1:4" ht="27.75" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:4" ht="27" x14ac:dyDescent="0.45">
       <c r="A10" s="2" t="s">
         <v>59</v>
       </c>
@@ -2121,7 +2149,7 @@
       </c>
       <c r="D10" s="3"/>
     </row>
-    <row r="11" spans="1:4" ht="27.75" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:4" ht="27" x14ac:dyDescent="0.45">
       <c r="A11" s="2" t="s">
         <v>59</v>
       </c>
@@ -2133,7 +2161,7 @@
       </c>
       <c r="D11" s="3"/>
     </row>
-    <row r="12" spans="1:4" ht="27.75" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:4" ht="27" x14ac:dyDescent="0.45">
       <c r="A12" s="2" t="s">
         <v>59</v>
       </c>
@@ -2145,7 +2173,7 @@
       </c>
       <c r="D12" s="3"/>
     </row>
-    <row r="13" spans="1:4" ht="27.75" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:4" ht="27" x14ac:dyDescent="0.45">
       <c r="A13" s="2" t="s">
         <v>61</v>
       </c>
@@ -2157,7 +2185,7 @@
       </c>
       <c r="D13" s="3"/>
     </row>
-    <row r="14" spans="1:4" ht="27.75" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:4" ht="27" x14ac:dyDescent="0.45">
       <c r="A14" s="2" t="s">
         <v>61</v>
       </c>
@@ -2169,7 +2197,7 @@
       </c>
       <c r="D14" s="3"/>
     </row>
-    <row r="15" spans="1:4" ht="54" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:4" ht="27" x14ac:dyDescent="0.45">
       <c r="A15" s="2" t="s">
         <v>93</v>
       </c>
@@ -2205,7 +2233,7 @@
       </c>
       <c r="D17" s="3"/>
     </row>
-    <row r="18" spans="1:4" ht="27.75" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:4" ht="27" x14ac:dyDescent="0.45">
       <c r="A18" s="2" t="s">
         <v>100</v>
       </c>
@@ -2217,7 +2245,7 @@
       </c>
       <c r="D18" s="3"/>
     </row>
-    <row r="19" spans="1:4" ht="27.75" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:4" ht="27" x14ac:dyDescent="0.45">
       <c r="A19" s="2" t="s">
         <v>100</v>
       </c>
@@ -2229,7 +2257,7 @@
       </c>
       <c r="D19" s="3"/>
     </row>
-    <row r="20" spans="1:4" ht="40.5" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:4" ht="27" x14ac:dyDescent="0.45">
       <c r="A20" s="2" t="s">
         <v>100</v>
       </c>
@@ -2241,7 +2269,7 @@
       </c>
       <c r="D20" s="3"/>
     </row>
-    <row r="21" spans="1:4" ht="27.75" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:4" ht="27" x14ac:dyDescent="0.45">
       <c r="A21" s="2" t="s">
         <v>100</v>
       </c>
@@ -2253,7 +2281,7 @@
       </c>
       <c r="D21" s="3"/>
     </row>
-    <row r="22" spans="1:4" ht="54" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:4" ht="27" x14ac:dyDescent="0.45">
       <c r="A22" s="2" t="s">
         <v>107</v>
       </c>
@@ -2277,7 +2305,7 @@
       </c>
       <c r="D23" s="3"/>
     </row>
-    <row r="24" spans="1:4" ht="27" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A24" s="2" t="s">
         <v>107</v>
       </c>
@@ -2289,7 +2317,7 @@
       </c>
       <c r="D24" s="3"/>
     </row>
-    <row r="25" spans="1:4" ht="27.75" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:4" ht="27" x14ac:dyDescent="0.45">
       <c r="A25" s="2" t="s">
         <v>69</v>
       </c>
@@ -2301,7 +2329,7 @@
       </c>
       <c r="D25" s="3"/>
     </row>
-    <row r="26" spans="1:4" ht="27.75" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:4" ht="27" x14ac:dyDescent="0.45">
       <c r="A26" s="2" t="s">
         <v>69</v>
       </c>
@@ -2313,7 +2341,7 @@
       </c>
       <c r="D26" s="3"/>
     </row>
-    <row r="27" spans="1:4" ht="40.5" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:4" ht="27" x14ac:dyDescent="0.45">
       <c r="A27" s="2" t="s">
         <v>69</v>
       </c>
@@ -2325,7 +2353,7 @@
       </c>
       <c r="D27" s="3"/>
     </row>
-    <row r="28" spans="1:4" ht="40.5" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:4" ht="27" x14ac:dyDescent="0.45">
       <c r="A28" s="2" t="s">
         <v>69</v>
       </c>
@@ -2337,7 +2365,7 @@
       </c>
       <c r="D28" s="3"/>
     </row>
-    <row r="29" spans="1:4" ht="27.75" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:4" ht="27" x14ac:dyDescent="0.45">
       <c r="A29" s="2" t="s">
         <v>69</v>
       </c>
@@ -2788,8 +2816,11 @@
       <c r="B17" t="s">
         <v>186</v>
       </c>
-      <c r="C17">
+      <c r="C17" s="6">
         <v>7</v>
+      </c>
+      <c r="D17" t="s">
+        <v>207</v>
       </c>
       <c r="F17" t="s">
         <v>187</v>
@@ -2816,8 +2847,11 @@
       <c r="B19" t="s">
         <v>187</v>
       </c>
-      <c r="C19">
+      <c r="C19" s="6">
         <v>5</v>
+      </c>
+      <c r="D19" t="s">
+        <v>210</v>
       </c>
       <c r="F19" t="s">
         <v>186</v>
@@ -2830,8 +2864,11 @@
       <c r="B20" t="s">
         <v>188</v>
       </c>
-      <c r="C20">
+      <c r="C20" s="6">
         <v>3</v>
+      </c>
+      <c r="D20" t="s">
+        <v>209</v>
       </c>
       <c r="F20" t="s">
         <v>191</v>
@@ -2844,8 +2881,11 @@
       <c r="B21" t="s">
         <v>189</v>
       </c>
-      <c r="C21">
+      <c r="C21" s="6">
         <v>1</v>
+      </c>
+      <c r="D21" t="s">
+        <v>206</v>
       </c>
       <c r="F21" t="s">
         <v>190</v>
@@ -2858,8 +2898,11 @@
       <c r="B22" t="s">
         <v>190</v>
       </c>
-      <c r="C22">
+      <c r="C22" s="6">
         <v>18</v>
+      </c>
+      <c r="D22" t="s">
+        <v>212</v>
       </c>
       <c r="F22" t="s">
         <v>193</v>
@@ -2872,8 +2915,11 @@
       <c r="B23" t="s">
         <v>191</v>
       </c>
-      <c r="C23">
+      <c r="C23" s="6">
         <v>11</v>
+      </c>
+      <c r="D23" t="s">
+        <v>208</v>
       </c>
       <c r="F23" t="s">
         <v>204</v>
@@ -2886,8 +2932,11 @@
       <c r="B24" t="s">
         <v>192</v>
       </c>
-      <c r="C24">
+      <c r="C24" s="6">
         <v>6</v>
+      </c>
+      <c r="D24" t="s">
+        <v>211</v>
       </c>
       <c r="F24" t="s">
         <v>184</v>

</xml_diff>

<commit_message>
Deployed f8db4c8 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/NSI_Premiere/Classeur1.xlsx
+++ b/NSI_Premiere/Classeur1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\--- LYCEE ---\ENSEIGNEMENT_G\docs\NSI_Premiere\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{372F3D1D-9786-49D3-8E2A-AC0827F8B947}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB1BB214-CD60-4539-BCB6-AFA0854A76F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10718" yWindow="0" windowWidth="10965" windowHeight="12863" activeTab="4" xr2:uid="{C3D69442-6D2C-43E5-8165-E9BA2FDD5BB6}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="221">
   <si>
     <r>
       <t>ThèmeContenus (Compétence)Capacités attendues &amp; CommentairesN° Activité</t>
@@ -989,6 +989,30 @@
   </si>
   <si>
     <t>LP07</t>
+  </si>
+  <si>
+    <t>Cours</t>
+  </si>
+  <si>
+    <t>Synthese</t>
+  </si>
+  <si>
+    <t>Flashcard</t>
+  </si>
+  <si>
+    <t>Quiz</t>
+  </si>
+  <si>
+    <t>Exercices</t>
+  </si>
+  <si>
+    <t>Activité</t>
+  </si>
+  <si>
+    <t>LP08</t>
+  </si>
+  <si>
+    <t>avant dico</t>
   </si>
 </sst>
 </file>
@@ -1058,7 +1082,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1074,6 +1098,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment textRotation="90"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2703,19 +2730,42 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{620BD464-A307-46DA-B24A-241C5ED06F30}">
-  <dimension ref="B5:G35"/>
+  <dimension ref="B4:N34"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="52.53125" customWidth="1"/>
-    <col min="6" max="6" width="36.265625" customWidth="1"/>
+    <col min="5" max="12" width="2.86328125" customWidth="1"/>
+    <col min="13" max="13" width="36.265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:14" ht="96.4" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E4" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>216</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="J4" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="K4" s="7"/>
+      <c r="L4" s="7"/>
+    </row>
+    <row r="5" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B5" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="6" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B6" t="s">
         <v>175</v>
       </c>
@@ -2723,7 +2773,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B7" t="s">
         <v>176</v>
       </c>
@@ -2731,7 +2781,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B8" t="s">
         <v>177</v>
       </c>
@@ -2739,7 +2789,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B9" t="s">
         <v>178</v>
       </c>
@@ -2747,7 +2797,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="10" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B10" t="s">
         <v>179</v>
       </c>
@@ -2755,7 +2805,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="11" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B11" t="s">
         <v>180</v>
       </c>
@@ -2763,7 +2813,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="12" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B12" t="s">
         <v>181</v>
       </c>
@@ -2771,7 +2821,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B13" t="s">
         <v>182</v>
       </c>
@@ -2779,40 +2829,40 @@
         <v>205</v>
       </c>
     </row>
-    <row r="14" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="14" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B14" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="15" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="15" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B15" t="s">
         <v>184</v>
       </c>
       <c r="C15">
         <v>26</v>
       </c>
-      <c r="F15" t="s">
+      <c r="M15" t="s">
         <v>189</v>
       </c>
-      <c r="G15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="2:7" x14ac:dyDescent="0.45">
+      <c r="N15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B16" t="s">
         <v>185</v>
       </c>
       <c r="C16">
         <v>27</v>
       </c>
-      <c r="F16" t="s">
+      <c r="M16" t="s">
         <v>188</v>
       </c>
-      <c r="G16">
+      <c r="N16">
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="17" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B17" t="s">
         <v>186</v>
       </c>
@@ -2822,223 +2872,374 @@
       <c r="D17" t="s">
         <v>207</v>
       </c>
-      <c r="F17" t="s">
+      <c r="E17">
+        <v>1</v>
+      </c>
+      <c r="F17">
+        <v>1</v>
+      </c>
+      <c r="G17">
+        <v>1</v>
+      </c>
+      <c r="H17">
+        <v>1</v>
+      </c>
+      <c r="I17">
+        <v>2</v>
+      </c>
+      <c r="J17">
+        <v>0</v>
+      </c>
+      <c r="M17" t="s">
         <v>187</v>
       </c>
-      <c r="G17">
+      <c r="N17">
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="18" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B18" t="s">
+        <v>187</v>
+      </c>
+      <c r="C18" s="6">
+        <v>5</v>
+      </c>
+      <c r="D18" t="s">
+        <v>210</v>
+      </c>
+      <c r="E18">
+        <v>1</v>
+      </c>
+      <c r="F18">
+        <v>1</v>
+      </c>
+      <c r="G18">
+        <v>1</v>
+      </c>
+      <c r="H18">
+        <v>1</v>
+      </c>
+      <c r="I18">
+        <v>3</v>
+      </c>
+      <c r="J18">
+        <v>2</v>
+      </c>
+      <c r="M18" t="s">
+        <v>192</v>
+      </c>
+      <c r="N18">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="B19" t="s">
+        <v>188</v>
+      </c>
+      <c r="C19" s="6">
+        <v>3</v>
+      </c>
+      <c r="D19" t="s">
+        <v>209</v>
+      </c>
+      <c r="E19">
+        <v>1</v>
+      </c>
+      <c r="F19">
+        <v>1</v>
+      </c>
+      <c r="G19">
+        <v>1</v>
+      </c>
+      <c r="H19">
+        <v>1</v>
+      </c>
+      <c r="I19">
+        <v>2</v>
+      </c>
+      <c r="J19">
+        <v>1</v>
+      </c>
+      <c r="M19" t="s">
+        <v>186</v>
+      </c>
+      <c r="N19">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="B20" t="s">
+        <v>189</v>
+      </c>
+      <c r="C20" s="6">
+        <v>1</v>
+      </c>
+      <c r="D20" t="s">
+        <v>206</v>
+      </c>
+      <c r="E20">
+        <v>1</v>
+      </c>
+      <c r="F20">
+        <v>1</v>
+      </c>
+      <c r="G20">
+        <v>1</v>
+      </c>
+      <c r="H20">
+        <v>1</v>
+      </c>
+      <c r="I20">
+        <v>2</v>
+      </c>
+      <c r="J20">
+        <v>1</v>
+      </c>
+      <c r="M20" t="s">
+        <v>191</v>
+      </c>
+      <c r="N20">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="21" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="B21" t="s">
+        <v>190</v>
+      </c>
+      <c r="C21" s="6">
+        <v>18</v>
+      </c>
+      <c r="D21" t="s">
+        <v>212</v>
+      </c>
+      <c r="E21">
+        <v>1</v>
+      </c>
+      <c r="F21">
+        <v>1</v>
+      </c>
+      <c r="G21">
+        <v>1</v>
+      </c>
+      <c r="H21">
+        <v>1</v>
+      </c>
+      <c r="I21">
+        <v>3</v>
+      </c>
+      <c r="J21">
+        <v>2</v>
+      </c>
+      <c r="M21" t="s">
+        <v>190</v>
+      </c>
+      <c r="N21">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="22" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="B22" t="s">
+        <v>191</v>
+      </c>
+      <c r="C22" s="6">
+        <v>11</v>
+      </c>
+      <c r="D22" t="s">
+        <v>208</v>
+      </c>
+      <c r="E22">
+        <v>1</v>
+      </c>
+      <c r="F22">
+        <v>1</v>
+      </c>
+      <c r="G22">
+        <v>1</v>
+      </c>
+      <c r="H22">
+        <v>1</v>
+      </c>
+      <c r="I22">
+        <v>1</v>
+      </c>
+      <c r="J22">
+        <v>1</v>
+      </c>
+      <c r="M22" t="s">
+        <v>193</v>
+      </c>
+      <c r="N22">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="B23" t="s">
+        <v>192</v>
+      </c>
+      <c r="C23" s="6">
+        <v>6</v>
+      </c>
+      <c r="D23" t="s">
+        <v>211</v>
+      </c>
+      <c r="E23">
+        <v>1</v>
+      </c>
+      <c r="F23">
+        <v>1</v>
+      </c>
+      <c r="G23">
+        <v>1</v>
+      </c>
+      <c r="H23">
+        <v>1</v>
+      </c>
+      <c r="I23">
+        <v>3</v>
+      </c>
+      <c r="J23">
+        <v>2</v>
+      </c>
+      <c r="M23" t="s">
         <v>204</v>
       </c>
-      <c r="C18">
+      <c r="N23">
         <v>24</v>
       </c>
-      <c r="F18" t="s">
-        <v>192</v>
-      </c>
-      <c r="G18">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="19" spans="2:7" x14ac:dyDescent="0.45">
-      <c r="B19" t="s">
-        <v>187</v>
-      </c>
-      <c r="C19" s="6">
-        <v>5</v>
-      </c>
-      <c r="D19" t="s">
-        <v>210</v>
-      </c>
-      <c r="F19" t="s">
-        <v>186</v>
-      </c>
-      <c r="G19">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="20" spans="2:7" x14ac:dyDescent="0.45">
-      <c r="B20" t="s">
-        <v>188</v>
-      </c>
-      <c r="C20" s="6">
-        <v>3</v>
-      </c>
-      <c r="D20" t="s">
-        <v>209</v>
-      </c>
-      <c r="F20" t="s">
-        <v>191</v>
-      </c>
-      <c r="G20">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="21" spans="2:7" x14ac:dyDescent="0.45">
-      <c r="B21" t="s">
-        <v>189</v>
-      </c>
-      <c r="C21" s="6">
-        <v>1</v>
-      </c>
-      <c r="D21" t="s">
-        <v>206</v>
-      </c>
-      <c r="F21" t="s">
-        <v>190</v>
-      </c>
-      <c r="G21">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="22" spans="2:7" x14ac:dyDescent="0.45">
-      <c r="B22" t="s">
-        <v>190</v>
-      </c>
-      <c r="C22" s="6">
-        <v>18</v>
-      </c>
-      <c r="D22" t="s">
-        <v>212</v>
-      </c>
-      <c r="F22" t="s">
+    </row>
+    <row r="24" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="B24" t="s">
         <v>193</v>
       </c>
-      <c r="G22">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="23" spans="2:7" x14ac:dyDescent="0.45">
-      <c r="B23" t="s">
-        <v>191</v>
-      </c>
-      <c r="C23" s="6">
-        <v>11</v>
-      </c>
-      <c r="D23" t="s">
-        <v>208</v>
-      </c>
-      <c r="F23" t="s">
-        <v>204</v>
-      </c>
-      <c r="G23">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="24" spans="2:7" x14ac:dyDescent="0.45">
-      <c r="B24" t="s">
-        <v>192</v>
-      </c>
-      <c r="C24" s="6">
-        <v>6</v>
+      <c r="C24" t="s">
+        <v>220</v>
       </c>
       <c r="D24" t="s">
-        <v>211</v>
-      </c>
-      <c r="F24" t="s">
+        <v>219</v>
+      </c>
+      <c r="E24">
+        <v>1</v>
+      </c>
+      <c r="F24">
+        <v>1</v>
+      </c>
+      <c r="G24">
+        <v>1</v>
+      </c>
+      <c r="H24">
+        <v>1</v>
+      </c>
+      <c r="M24" t="s">
         <v>184</v>
       </c>
-      <c r="G24">
+      <c r="N24">
         <v>26</v>
       </c>
     </row>
-    <row r="25" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="25" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B25" t="s">
-        <v>193</v>
-      </c>
-      <c r="C25">
-        <v>21</v>
-      </c>
-      <c r="F25" t="s">
+        <v>194</v>
+      </c>
+      <c r="M25" t="s">
         <v>185</v>
       </c>
-      <c r="G25">
+      <c r="N25">
         <v>27</v>
       </c>
     </row>
-    <row r="26" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="26" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B26" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="27" spans="2:7" x14ac:dyDescent="0.45">
+        <v>195</v>
+      </c>
+      <c r="C26">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B27" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C27">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="28" spans="2:7" x14ac:dyDescent="0.45">
+        <v>2</v>
+      </c>
+      <c r="E27">
+        <v>1</v>
+      </c>
+      <c r="G27">
+        <v>1</v>
+      </c>
+      <c r="H27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B28" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C28">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="29" spans="2:7" x14ac:dyDescent="0.45">
+        <v>8</v>
+      </c>
+      <c r="E28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B29" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C29">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="30" spans="2:7" x14ac:dyDescent="0.45">
+        <v>9</v>
+      </c>
+      <c r="E29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B30" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C30">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="31" spans="2:7" x14ac:dyDescent="0.45">
+        <v>10</v>
+      </c>
+      <c r="E30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B31" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C31">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="32" spans="2:7" x14ac:dyDescent="0.45">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="32" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B32" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C32">
-        <v>23</v>
+        <v>19</v>
       </c>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.45">
       <c r="B33" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C33">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="34" spans="2:3" x14ac:dyDescent="0.45">
       <c r="B34" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C34">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="35" spans="2:3" x14ac:dyDescent="0.45">
-      <c r="B35" t="s">
-        <v>203</v>
-      </c>
-      <c r="C35">
         <v>22</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="F15:G25">
-    <sortCondition ref="G15:G25"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="M15:N25">
+    <sortCondition ref="N15:N25"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Deployed a89e246 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/NSI_Premiere/Classeur1.xlsx
+++ b/NSI_Premiere/Classeur1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\--- LYCEE ---\ENSEIGNEMENT_G\docs\NSI_Premiere\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB1BB214-CD60-4539-BCB6-AFA0854A76F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D160A94-B48B-4C56-A52E-9068CE75883C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="4" xr2:uid="{C3D69442-6D2C-43E5-8165-E9BA2FDD5BB6}"/>
+    <workbookView xWindow="10718" yWindow="0" windowWidth="10965" windowHeight="12863" activeTab="4" xr2:uid="{C3D69442-6D2C-43E5-8165-E9BA2FDD5BB6}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="226">
   <si>
     <r>
       <t>ThèmeContenus (Compétence)Capacités attendues &amp; CommentairesN° Activité</t>
@@ -1013,6 +1013,21 @@
   </si>
   <si>
     <t>avant dico</t>
+  </si>
+  <si>
+    <t>RD01</t>
+  </si>
+  <si>
+    <t>RD02</t>
+  </si>
+  <si>
+    <t>RD03</t>
+  </si>
+  <si>
+    <t>RD04</t>
+  </si>
+  <si>
+    <t>RD05</t>
   </si>
 </sst>
 </file>
@@ -2733,7 +2748,7 @@
   <dimension ref="B4:N34"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="52.53125" customWidth="1"/>
+    <col min="2" max="2" width="35.265625" customWidth="1"/>
     <col min="5" max="12" width="2.86328125" customWidth="1"/>
     <col min="13" max="13" width="36.265625" customWidth="1"/>
   </cols>
@@ -3154,6 +3169,9 @@
       <c r="C26">
         <v>4</v>
       </c>
+      <c r="D26" t="s">
+        <v>222</v>
+      </c>
     </row>
     <row r="27" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B27" t="s">
@@ -3162,6 +3180,9 @@
       <c r="C27">
         <v>2</v>
       </c>
+      <c r="D27" t="s">
+        <v>221</v>
+      </c>
       <c r="E27">
         <v>1</v>
       </c>
@@ -3169,6 +3190,12 @@
         <v>1</v>
       </c>
       <c r="H27">
+        <v>1</v>
+      </c>
+      <c r="I27">
+        <v>1</v>
+      </c>
+      <c r="J27">
         <v>1</v>
       </c>
     </row>
@@ -3179,7 +3206,13 @@
       <c r="C28">
         <v>8</v>
       </c>
+      <c r="D28" t="s">
+        <v>223</v>
+      </c>
       <c r="E28">
+        <v>1</v>
+      </c>
+      <c r="J28">
         <v>1</v>
       </c>
     </row>
@@ -3190,6 +3223,9 @@
       <c r="C29">
         <v>9</v>
       </c>
+      <c r="D29" t="s">
+        <v>224</v>
+      </c>
       <c r="E29">
         <v>1</v>
       </c>
@@ -3201,7 +3237,13 @@
       <c r="C30">
         <v>10</v>
       </c>
+      <c r="D30" t="s">
+        <v>225</v>
+      </c>
       <c r="E30">
+        <v>1</v>
+      </c>
+      <c r="J30">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed cff4140 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/NSI_Premiere/Classeur1.xlsx
+++ b/NSI_Premiere/Classeur1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\--- LYCEE ---\ENSEIGNEMENT_G\docs\NSI_Premiere\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D160A94-B48B-4C56-A52E-9068CE75883C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7564C3E2-7851-405D-90FD-DE1872EAA41E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10718" yWindow="0" windowWidth="10965" windowHeight="12863" activeTab="4" xr2:uid="{C3D69442-6D2C-43E5-8165-E9BA2FDD5BB6}"/>
   </bookViews>
@@ -3213,7 +3213,7 @@
         <v>1</v>
       </c>
       <c r="J28">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29" spans="2:14" x14ac:dyDescent="0.45">
@@ -3227,6 +3227,9 @@
         <v>224</v>
       </c>
       <c r="E29">
+        <v>1</v>
+      </c>
+      <c r="J29">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed 8636c87 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/NSI_Premiere/Classeur1.xlsx
+++ b/NSI_Premiere/Classeur1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\--- LYCEE ---\ENSEIGNEMENT_G\docs\NSI_Premiere\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7564C3E2-7851-405D-90FD-DE1872EAA41E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{367AACEC-60EB-4762-A3BA-CD0FFA27B512}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10718" yWindow="0" windowWidth="10965" windowHeight="12863" activeTab="4" xr2:uid="{C3D69442-6D2C-43E5-8165-E9BA2FDD5BB6}"/>
   </bookViews>
@@ -3172,6 +3172,9 @@
       <c r="D26" t="s">
         <v>222</v>
       </c>
+      <c r="E26">
+        <v>1</v>
+      </c>
     </row>
     <row r="27" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B27" t="s">

</xml_diff>

<commit_message>
Deployed 5c372f2 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/NSI_Premiere/Classeur1.xlsx
+++ b/NSI_Premiere/Classeur1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\--- LYCEE ---\ENSEIGNEMENT_G\docs\NSI_Premiere\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{367AACEC-60EB-4762-A3BA-CD0FFA27B512}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18196668-3282-400F-9F6F-58BF631F0165}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10718" yWindow="0" windowWidth="10965" windowHeight="12863" activeTab="4" xr2:uid="{C3D69442-6D2C-43E5-8165-E9BA2FDD5BB6}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="4" xr2:uid="{C3D69442-6D2C-43E5-8165-E9BA2FDD5BB6}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="225">
   <si>
     <r>
       <t>ThèmeContenus (Compétence)Capacités attendues &amp; CommentairesN° Activité</t>
@@ -952,18 +952,6 @@
     <t xml:space="preserve">    ├───RD_Representation_Texte</t>
   </si>
   <si>
-    <t xml:space="preserve">    ├───RD_Tables_Fusion</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    ├───RD_Tables_Indexation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    ├───RD_Tables_Recherche</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    └───RD_Tables_Tri</t>
-  </si>
-  <si>
     <t>│   ├───LP_Algos_recherche (Dichotomie)</t>
   </si>
   <si>
@@ -1028,6 +1016,15 @@
   </si>
   <si>
     <t>RD05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    ├───RD_Tables</t>
+  </si>
+  <si>
+    <t>AF: import de fichier texte + recherche</t>
+  </si>
+  <si>
+    <t>X</t>
   </si>
 </sst>
 </file>
@@ -2745,42 +2742,44 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{620BD464-A307-46DA-B24A-241C5ED06F30}">
-  <dimension ref="B4:N34"/>
+  <dimension ref="B4:O31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="35.265625" customWidth="1"/>
     <col min="5" max="12" width="2.86328125" customWidth="1"/>
-    <col min="13" max="13" width="36.265625" customWidth="1"/>
+    <col min="13" max="13" width="21" customWidth="1"/>
+    <col min="14" max="14" width="36.265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="2:14" ht="96.4" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:15" ht="96.4" customHeight="1" x14ac:dyDescent="0.45">
       <c r="E4" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>211</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="I4" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="J4" s="7" t="s">
         <v>214</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>215</v>
-      </c>
-      <c r="H4" s="7" t="s">
-        <v>216</v>
-      </c>
-      <c r="I4" s="7" t="s">
-        <v>217</v>
-      </c>
-      <c r="J4" s="7" t="s">
-        <v>218</v>
       </c>
       <c r="K4" s="7"/>
       <c r="L4" s="7"/>
-    </row>
-    <row r="5" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="M4" s="7"/>
+    </row>
+    <row r="5" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B5" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="6" spans="2:14" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B6" t="s">
         <v>175</v>
       </c>
@@ -2788,7 +2787,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="2:14" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B7" t="s">
         <v>176</v>
       </c>
@@ -2796,7 +2795,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="2:14" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B8" t="s">
         <v>177</v>
       </c>
@@ -2804,7 +2803,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="2:14" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B9" t="s">
         <v>178</v>
       </c>
@@ -2812,7 +2811,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="2:14" x14ac:dyDescent="0.45">
+    <row r="10" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B10" t="s">
         <v>179</v>
       </c>
@@ -2820,7 +2819,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="2:14" x14ac:dyDescent="0.45">
+    <row r="11" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B11" t="s">
         <v>180</v>
       </c>
@@ -2828,7 +2827,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="2:14" x14ac:dyDescent="0.45">
+    <row r="12" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B12" t="s">
         <v>181</v>
       </c>
@@ -2836,48 +2835,48 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="2:14" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B13" t="s">
         <v>182</v>
       </c>
       <c r="C13" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="14" spans="2:14" x14ac:dyDescent="0.45">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="14" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B14" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="15" spans="2:14" x14ac:dyDescent="0.45">
+    <row r="15" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B15" t="s">
         <v>184</v>
       </c>
       <c r="C15">
         <v>26</v>
       </c>
-      <c r="M15" t="s">
+      <c r="N15" t="s">
         <v>189</v>
       </c>
-      <c r="N15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="O15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B16" t="s">
         <v>185</v>
       </c>
       <c r="C16">
         <v>27</v>
       </c>
-      <c r="M16" t="s">
+      <c r="N16" t="s">
         <v>188</v>
       </c>
-      <c r="N16">
+      <c r="O16">
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="2:14" x14ac:dyDescent="0.45">
+    <row r="17" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B17" t="s">
         <v>186</v>
       </c>
@@ -2885,7 +2884,7 @@
         <v>7</v>
       </c>
       <c r="D17" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="E17">
         <v>1</v>
@@ -2905,14 +2904,14 @@
       <c r="J17">
         <v>0</v>
       </c>
-      <c r="M17" t="s">
+      <c r="N17" t="s">
         <v>187</v>
       </c>
-      <c r="N17">
+      <c r="O17">
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="2:14" x14ac:dyDescent="0.45">
+    <row r="18" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B18" t="s">
         <v>187</v>
       </c>
@@ -2920,7 +2919,7 @@
         <v>5</v>
       </c>
       <c r="D18" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="E18">
         <v>1</v>
@@ -2940,14 +2939,14 @@
       <c r="J18">
         <v>2</v>
       </c>
-      <c r="M18" t="s">
+      <c r="N18" t="s">
         <v>192</v>
       </c>
-      <c r="N18">
+      <c r="O18">
         <v>6</v>
       </c>
     </row>
-    <row r="19" spans="2:14" x14ac:dyDescent="0.45">
+    <row r="19" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B19" t="s">
         <v>188</v>
       </c>
@@ -2955,7 +2954,7 @@
         <v>3</v>
       </c>
       <c r="D19" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="E19">
         <v>1</v>
@@ -2975,14 +2974,14 @@
       <c r="J19">
         <v>1</v>
       </c>
-      <c r="M19" t="s">
+      <c r="N19" t="s">
         <v>186</v>
       </c>
-      <c r="N19">
+      <c r="O19">
         <v>7</v>
       </c>
     </row>
-    <row r="20" spans="2:14" x14ac:dyDescent="0.45">
+    <row r="20" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B20" t="s">
         <v>189</v>
       </c>
@@ -2990,7 +2989,7 @@
         <v>1</v>
       </c>
       <c r="D20" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="E20">
         <v>1</v>
@@ -3010,14 +3009,14 @@
       <c r="J20">
         <v>1</v>
       </c>
-      <c r="M20" t="s">
+      <c r="N20" t="s">
         <v>191</v>
       </c>
-      <c r="N20">
+      <c r="O20">
         <v>11</v>
       </c>
     </row>
-    <row r="21" spans="2:14" x14ac:dyDescent="0.45">
+    <row r="21" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B21" t="s">
         <v>190</v>
       </c>
@@ -3025,7 +3024,7 @@
         <v>18</v>
       </c>
       <c r="D21" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="E21">
         <v>1</v>
@@ -3045,14 +3044,14 @@
       <c r="J21">
         <v>2</v>
       </c>
-      <c r="M21" t="s">
+      <c r="N21" t="s">
         <v>190</v>
       </c>
-      <c r="N21">
+      <c r="O21">
         <v>18</v>
       </c>
     </row>
-    <row r="22" spans="2:14" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B22" t="s">
         <v>191</v>
       </c>
@@ -3060,7 +3059,7 @@
         <v>11</v>
       </c>
       <c r="D22" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="E22">
         <v>1</v>
@@ -3080,14 +3079,14 @@
       <c r="J22">
         <v>1</v>
       </c>
-      <c r="M22" t="s">
+      <c r="N22" t="s">
         <v>193</v>
       </c>
-      <c r="N22">
+      <c r="O22">
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="2:14" x14ac:dyDescent="0.45">
+    <row r="23" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B23" t="s">
         <v>192</v>
       </c>
@@ -3095,7 +3094,7 @@
         <v>6</v>
       </c>
       <c r="D23" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -3115,22 +3114,22 @@
       <c r="J23">
         <v>2</v>
       </c>
-      <c r="M23" t="s">
-        <v>204</v>
-      </c>
-      <c r="N23">
+      <c r="N23" t="s">
+        <v>200</v>
+      </c>
+      <c r="O23">
         <v>24</v>
       </c>
     </row>
-    <row r="24" spans="2:14" x14ac:dyDescent="0.45">
+    <row r="24" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B24" t="s">
         <v>193</v>
       </c>
       <c r="C24" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="D24" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="E24">
         <v>1</v>
@@ -3144,25 +3143,25 @@
       <c r="H24">
         <v>1</v>
       </c>
-      <c r="M24" t="s">
+      <c r="N24" t="s">
         <v>184</v>
       </c>
-      <c r="N24">
+      <c r="O24">
         <v>26</v>
       </c>
     </row>
-    <row r="25" spans="2:14" x14ac:dyDescent="0.45">
+    <row r="25" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B25" t="s">
         <v>194</v>
       </c>
-      <c r="M25" t="s">
+      <c r="N25" t="s">
         <v>185</v>
       </c>
-      <c r="N25">
+      <c r="O25">
         <v>27</v>
       </c>
     </row>
-    <row r="26" spans="2:14" x14ac:dyDescent="0.45">
+    <row r="26" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B26" t="s">
         <v>195</v>
       </c>
@@ -3170,13 +3169,19 @@
         <v>4</v>
       </c>
       <c r="D26" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="E26">
         <v>1</v>
       </c>
-    </row>
-    <row r="27" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="I26">
+        <v>1</v>
+      </c>
+      <c r="J26" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="27" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B27" t="s">
         <v>196</v>
       </c>
@@ -3184,7 +3189,7 @@
         <v>2</v>
       </c>
       <c r="D27" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="E27">
         <v>1</v>
@@ -3202,7 +3207,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="2:14" x14ac:dyDescent="0.45">
+    <row r="28" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B28" t="s">
         <v>197</v>
       </c>
@@ -3210,16 +3215,19 @@
         <v>8</v>
       </c>
       <c r="D28" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="E28">
         <v>1</v>
       </c>
+      <c r="I28">
+        <v>1</v>
+      </c>
       <c r="J28">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="29" spans="2:14" x14ac:dyDescent="0.45">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B29" t="s">
         <v>198</v>
       </c>
@@ -3227,16 +3235,13 @@
         <v>9</v>
       </c>
       <c r="D29" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="E29">
         <v>1</v>
       </c>
-      <c r="J29">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30" spans="2:14" x14ac:dyDescent="0.45">
+    </row>
+    <row r="30" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B30" t="s">
         <v>199</v>
       </c>
@@ -3244,7 +3249,7 @@
         <v>10</v>
       </c>
       <c r="D30" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="E30">
         <v>1</v>
@@ -3252,42 +3257,27 @@
       <c r="J30">
         <v>1</v>
       </c>
-    </row>
-    <row r="31" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="N30" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="31" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B31" t="s">
-        <v>200</v>
+        <v>222</v>
       </c>
       <c r="C31">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="32" spans="2:14" x14ac:dyDescent="0.45">
-      <c r="B32" t="s">
-        <v>201</v>
-      </c>
-      <c r="C32">
         <v>19</v>
       </c>
-    </row>
-    <row r="33" spans="2:3" x14ac:dyDescent="0.45">
-      <c r="B33" t="s">
-        <v>202</v>
-      </c>
-      <c r="C33">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="34" spans="2:3" x14ac:dyDescent="0.45">
-      <c r="B34" t="s">
-        <v>203</v>
-      </c>
-      <c r="C34">
-        <v>22</v>
+      <c r="E31">
+        <v>1</v>
+      </c>
+      <c r="J31">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="M15:N25">
-    <sortCondition ref="N15:N25"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="N15:O25">
+    <sortCondition ref="O15:O25"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Deployed c0e3efa with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/NSI_Premiere/Classeur1.xlsx
+++ b/NSI_Premiere/Classeur1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\--- LYCEE ---\ENSEIGNEMENT_G\docs\NSI_Premiere\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18196668-3282-400F-9F6F-58BF631F0165}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16E2ACC8-A9B1-4538-95EE-910EF5FF7CA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="4" xr2:uid="{C3D69442-6D2C-43E5-8165-E9BA2FDD5BB6}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="5" xr2:uid="{C3D69442-6D2C-43E5-8165-E9BA2FDD5BB6}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="Feuil3" sheetId="3" r:id="rId3"/>
     <sheet name="Feuil4" sheetId="4" r:id="rId4"/>
     <sheet name="Feuil5" sheetId="5" r:id="rId5"/>
+    <sheet name="Feuil6" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="244">
   <si>
     <r>
       <t>ThèmeContenus (Compétence)Capacités attendues &amp; CommentairesN° Activité</t>
@@ -892,15 +893,6 @@
     <t>│   ├───_ARSE_Web_HTML01</t>
   </si>
   <si>
-    <t>│   ├───_ARSE_Web_HTML02</t>
-  </si>
-  <si>
-    <t>│   ├───_ARSE_Web_HTML03</t>
-  </si>
-  <si>
-    <t>│   └───_ARSE_Web_Interaction_Client_Serveur</t>
-  </si>
-  <si>
     <t>_LP_Langage_Programmation</t>
   </si>
   <si>
@@ -1025,6 +1017,72 @@
   </si>
   <si>
     <t>X</t>
+  </si>
+  <si>
+    <t>_ARSE_Reseau_introcution</t>
+  </si>
+  <si>
+    <t>_ARSE Adresse IP</t>
+  </si>
+  <si>
+    <t>_ARSE_Protocole Internet</t>
+  </si>
+  <si>
+    <t>Session 1</t>
+  </si>
+  <si>
+    <t>Session 2</t>
+  </si>
+  <si>
+    <t>Session 3</t>
+  </si>
+  <si>
+    <t>Session 4</t>
+  </si>
+  <si>
+    <t>BELLION Myrddin</t>
+  </si>
+  <si>
+    <t>BENNAJIB Ikram</t>
+  </si>
+  <si>
+    <t>DARTIES Gabriel</t>
+  </si>
+  <si>
+    <t>FAWCETT Amélie</t>
+  </si>
+  <si>
+    <t>FRANCHUK Vitalii</t>
+  </si>
+  <si>
+    <t>KASSOUS Ilyan</t>
+  </si>
+  <si>
+    <t>LACAM--GONCALVES Julia</t>
+  </si>
+  <si>
+    <t>MONCHOUX Jolin</t>
+  </si>
+  <si>
+    <t>NERRAND Dimitri</t>
+  </si>
+  <si>
+    <t>OUSPANOV Kazbek</t>
+  </si>
+  <si>
+    <t>PATTENDEN Laura</t>
+  </si>
+  <si>
+    <t>PROUST Alexandre</t>
+  </si>
+  <si>
+    <t>PUTIGNANO Chiara</t>
+  </si>
+  <si>
+    <t>UKIEVA Mislina</t>
+  </si>
+  <si>
+    <t>YADAV Swastika</t>
   </si>
 </sst>
 </file>
@@ -1082,7 +1140,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1090,11 +1148,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1113,6 +1186,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment textRotation="90"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2753,22 +2827,22 @@
   <sheetData>
     <row r="4" spans="2:15" ht="96.4" customHeight="1" x14ac:dyDescent="0.45">
       <c r="E4" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>208</v>
+      </c>
+      <c r="H4" s="7" t="s">
         <v>209</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="I4" s="7" t="s">
         <v>210</v>
       </c>
-      <c r="G4" s="7" t="s">
+      <c r="J4" s="7" t="s">
         <v>211</v>
-      </c>
-      <c r="H4" s="7" t="s">
-        <v>212</v>
-      </c>
-      <c r="I4" s="7" t="s">
-        <v>213</v>
-      </c>
-      <c r="J4" s="7" t="s">
-        <v>214</v>
       </c>
       <c r="K4" s="7"/>
       <c r="L4" s="7"/>
@@ -2802,6 +2876,12 @@
       <c r="C8">
         <v>12</v>
       </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="J8">
+        <v>1</v>
+      </c>
     </row>
     <row r="9" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B9" t="s">
@@ -2821,42 +2901,57 @@
     </row>
     <row r="11" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B11" t="s">
-        <v>180</v>
+        <v>222</v>
       </c>
       <c r="C11">
         <v>14</v>
       </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
     </row>
     <row r="12" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B12" t="s">
-        <v>181</v>
+        <v>223</v>
       </c>
       <c r="C12">
         <v>15</v>
       </c>
+      <c r="E12">
+        <v>1</v>
+      </c>
+      <c r="J12">
+        <v>1</v>
+      </c>
     </row>
     <row r="13" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B13" t="s">
-        <v>182</v>
+        <v>224</v>
       </c>
       <c r="C13" t="s">
-        <v>201</v>
+        <v>198</v>
+      </c>
+      <c r="E13">
+        <v>1</v>
+      </c>
+      <c r="J13">
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B14" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="15" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B15" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="C15">
         <v>26</v>
       </c>
       <c r="N15" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="O15">
         <v>1</v>
@@ -2864,13 +2959,13 @@
     </row>
     <row r="16" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B16" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="C16">
         <v>27</v>
       </c>
       <c r="N16" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="O16">
         <v>3</v>
@@ -2878,13 +2973,13 @@
     </row>
     <row r="17" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B17" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="C17" s="6">
         <v>7</v>
       </c>
       <c r="D17" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="E17">
         <v>1</v>
@@ -2905,7 +3000,7 @@
         <v>0</v>
       </c>
       <c r="N17" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="O17">
         <v>5</v>
@@ -2913,13 +3008,13 @@
     </row>
     <row r="18" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B18" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="C18" s="6">
         <v>5</v>
       </c>
       <c r="D18" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="E18">
         <v>1</v>
@@ -2940,7 +3035,7 @@
         <v>2</v>
       </c>
       <c r="N18" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="O18">
         <v>6</v>
@@ -2948,13 +3043,13 @@
     </row>
     <row r="19" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B19" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="C19" s="6">
         <v>3</v>
       </c>
       <c r="D19" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="E19">
         <v>1</v>
@@ -2975,7 +3070,7 @@
         <v>1</v>
       </c>
       <c r="N19" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="O19">
         <v>7</v>
@@ -2983,13 +3078,13 @@
     </row>
     <row r="20" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B20" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="C20" s="6">
         <v>1</v>
       </c>
       <c r="D20" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="E20">
         <v>1</v>
@@ -3010,7 +3105,7 @@
         <v>1</v>
       </c>
       <c r="N20" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="O20">
         <v>11</v>
@@ -3018,13 +3113,13 @@
     </row>
     <row r="21" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B21" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="C21" s="6">
         <v>18</v>
       </c>
       <c r="D21" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="E21">
         <v>1</v>
@@ -3045,7 +3140,7 @@
         <v>2</v>
       </c>
       <c r="N21" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="O21">
         <v>18</v>
@@ -3053,13 +3148,13 @@
     </row>
     <row r="22" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B22" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="C22" s="6">
         <v>11</v>
       </c>
       <c r="D22" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="E22">
         <v>1</v>
@@ -3080,7 +3175,7 @@
         <v>1</v>
       </c>
       <c r="N22" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="O22">
         <v>21</v>
@@ -3088,13 +3183,13 @@
     </row>
     <row r="23" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B23" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="C23" s="6">
         <v>6</v>
       </c>
       <c r="D23" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -3115,7 +3210,7 @@
         <v>2</v>
       </c>
       <c r="N23" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="O23">
         <v>24</v>
@@ -3123,13 +3218,13 @@
     </row>
     <row r="24" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B24" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="C24" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="D24" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="E24">
         <v>1</v>
@@ -3144,7 +3239,7 @@
         <v>1</v>
       </c>
       <c r="N24" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="O24">
         <v>26</v>
@@ -3152,10 +3247,10 @@
     </row>
     <row r="25" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B25" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="N25" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="O25">
         <v>27</v>
@@ -3163,13 +3258,13 @@
     </row>
     <row r="26" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B26" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="C26">
         <v>4</v>
       </c>
       <c r="D26" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="E26">
         <v>1</v>
@@ -3178,18 +3273,18 @@
         <v>1</v>
       </c>
       <c r="J26" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
     </row>
     <row r="27" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B27" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="C27">
         <v>2</v>
       </c>
       <c r="D27" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="E27">
         <v>1</v>
@@ -3209,13 +3304,13 @@
     </row>
     <row r="28" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B28" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="C28">
         <v>8</v>
       </c>
       <c r="D28" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="E28">
         <v>1</v>
@@ -3229,13 +3324,13 @@
     </row>
     <row r="29" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B29" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="C29">
         <v>9</v>
       </c>
       <c r="D29" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -3243,13 +3338,13 @@
     </row>
     <row r="30" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B30" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="C30">
         <v>10</v>
       </c>
       <c r="D30" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="E30">
         <v>1</v>
@@ -3258,12 +3353,12 @@
         <v>1</v>
       </c>
       <c r="N30" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
     </row>
     <row r="31" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B31" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="C31">
         <v>19</v>
@@ -3281,4 +3376,85 @@
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27B06C93-FCDE-4C7C-B0AD-5832CC1D02CA}">
+  <dimension ref="A4:D8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="4" width="15.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A4" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>226</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>227</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A5" s="8" t="s">
+        <v>240</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>229</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>233</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A6" s="8" t="s">
+        <v>243</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>234</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A7" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>231</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A8" s="8" t="s">
+        <v>235</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>239</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>242</v>
+      </c>
+      <c r="D8" s="8"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>